<commit_message>
Build prompt manager installers
</commit_message>
<xml_diff>
--- a/outputs/content-system-prompts/content-system-prompts-first-row.xlsx
+++ b/outputs/content-system-prompts/content-system-prompts-first-row.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt导入模板" sheetId="1" r:id="R3e2e00e4a4464109"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt导入模板" sheetId="1" r:id="R22978404c37d4cb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -273,7 +273,7 @@
 2. 每个切口必须包含：选题公式、推荐结构、时效判断、四维评分、标题方向、素材缺口。
 3. 四维评分包括：热爱程度、专业能力、市场需求、资源积累，每项 1-5 分。
 4. 优先推荐总分最高、最容易转成公众号观点文的切口。
-5. 输出必须能交给 content-brief-builder 继续生成 brief。</x:v>
+5. 输出必须能交给 content_outline_builder 继续生成文章大纲。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
         <x:v>选题,热点,上游决策</x:v>

</xml_diff>